<commit_message>
add 1 more survey, remove mean and SD scores
</commit_message>
<xml_diff>
--- a/surveyux/survey_eval.xlsx
+++ b/surveyux/survey_eval.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Githubs\IEEE-Technology-and-Society-Draft\surveyux\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0F6CCBD-4078-4FAF-837A-D0E163F2A4FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFB85949-586F-458B-98A9-4386BF0940BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30165" yWindow="2250" windowWidth="21600" windowHeight="11385" activeTab="1" xr2:uid="{D8488B4A-5A4F-4189-8080-6FE281BAE78B}"/>
+    <workbookView xWindow="31395" yWindow="1680" windowWidth="21600" windowHeight="11385" xr2:uid="{D8488B4A-5A4F-4189-8080-6FE281BAE78B}"/>
   </bookViews>
   <sheets>
     <sheet name="Likert Scale" sheetId="1" r:id="rId1"/>
@@ -243,12 +243,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -855,37 +854,64 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A12" s="3" t="s">
+      <c r="A12" t="s">
         <v>39</v>
       </c>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
-      <c r="I12" s="4"/>
-      <c r="J12" s="4"/>
+      <c r="B12" s="3">
+        <v>4</v>
+      </c>
+      <c r="C12" s="3">
+        <v>5</v>
+      </c>
+      <c r="D12" s="3">
+        <v>1</v>
+      </c>
+      <c r="E12" s="3">
+        <v>5</v>
+      </c>
+      <c r="F12" s="3">
+        <v>4</v>
+      </c>
+      <c r="G12" s="3">
+        <v>1</v>
+      </c>
+      <c r="H12" s="3">
+        <v>5</v>
+      </c>
+      <c r="I12" s="3">
+        <v>5</v>
+      </c>
+      <c r="J12" s="3">
+        <v>2</v>
+      </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A13" s="3" t="s">
+      <c r="A13" t="s">
         <v>40</v>
       </c>
-      <c r="B13" s="4"/>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
-      <c r="I13" s="4"/>
-      <c r="J13" s="4"/>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
+      <c r="J13" s="3"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>41</v>
       </c>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+      <c r="J14" s="3"/>
     </row>
     <row r="16" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
@@ -893,39 +919,39 @@
       </c>
       <c r="B16" s="2">
         <f>AVERAGE(B5:B14)</f>
-        <v>4.7142857142857144</v>
+        <v>4.625</v>
       </c>
       <c r="C16" s="2">
         <f t="shared" ref="C16:J16" si="0">AVERAGE(C5:C14)</f>
-        <v>4.5714285714285712</v>
+        <v>4.625</v>
       </c>
       <c r="D16" s="2">
         <f t="shared" si="0"/>
-        <v>1.8333333333333333</v>
+        <v>1.7142857142857142</v>
       </c>
       <c r="E16" s="2">
         <f t="shared" si="0"/>
-        <v>4.7142857142857144</v>
+        <v>4.75</v>
       </c>
       <c r="F16" s="2">
         <f t="shared" si="0"/>
-        <v>4.7142857142857144</v>
+        <v>4.625</v>
       </c>
       <c r="G16" s="2">
         <f t="shared" si="0"/>
-        <v>1.5714285714285714</v>
+        <v>1.5</v>
       </c>
       <c r="H16" s="2">
         <f t="shared" si="0"/>
-        <v>4.4285714285714288</v>
+        <v>4.5</v>
       </c>
       <c r="I16" s="2">
         <f t="shared" si="0"/>
-        <v>4.7142857142857144</v>
+        <v>4.75</v>
       </c>
       <c r="J16" s="2">
         <f t="shared" si="0"/>
-        <v>4.4285714285714288</v>
+        <v>4.125</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
@@ -934,39 +960,39 @@
       </c>
       <c r="B17" s="2">
         <f>_xlfn.STDEV.S(B5:B14)</f>
-        <v>0.48795003647426655</v>
+        <v>0.51754916950676566</v>
       </c>
       <c r="C17" s="2">
         <f t="shared" ref="C17:J17" si="1">_xlfn.STDEV.S(C5:C14)</f>
-        <v>0.53452248382485001</v>
+        <v>0.51754916950676566</v>
       </c>
       <c r="D17" s="2">
         <f t="shared" si="1"/>
-        <v>0.9831920802501749</v>
+        <v>0.95118973121134176</v>
       </c>
       <c r="E17" s="2">
         <f t="shared" si="1"/>
-        <v>0.48795003647426655</v>
+        <v>0.46291004988627571</v>
       </c>
       <c r="F17" s="2">
         <f t="shared" si="1"/>
-        <v>0.48795003647426655</v>
+        <v>0.51754916950676566</v>
       </c>
       <c r="G17" s="2">
         <f t="shared" si="1"/>
-        <v>0.7867957924694432</v>
+        <v>0.7559289460184544</v>
       </c>
       <c r="H17" s="2">
         <f t="shared" si="1"/>
-        <v>0.53452248382485001</v>
+        <v>0.53452248382484879</v>
       </c>
       <c r="I17" s="2">
         <f t="shared" si="1"/>
-        <v>0.48795003647426666</v>
+        <v>0.46291004988627571</v>
       </c>
       <c r="J17" s="2">
         <f t="shared" si="1"/>
-        <v>0.78679579246944398</v>
+        <v>1.1259916264596033</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add more results and discussion (survey)
</commit_message>
<xml_diff>
--- a/surveyux/survey_eval.xlsx
+++ b/surveyux/survey_eval.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Githubs\IEEE-Technology-and-Society-Draft\surveyux\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFB85949-586F-458B-98A9-4386BF0940BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66B0040B-3C9F-4803-A218-EF5876109909}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31395" yWindow="1680" windowWidth="21600" windowHeight="11385" xr2:uid="{D8488B4A-5A4F-4189-8080-6FE281BAE78B}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{D8488B4A-5A4F-4189-8080-6FE281BAE78B}"/>
   </bookViews>
   <sheets>
     <sheet name="Likert Scale" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="48">
   <si>
     <t>N = 7</t>
   </si>
@@ -189,6 +189,24 @@
   </si>
   <si>
     <t>P10</t>
+  </si>
+  <si>
+    <t>intuitive controls</t>
+  </si>
+  <si>
+    <t>faster response times (voice to motion)</t>
+  </si>
+  <si>
+    <t>multiple languages, interoperability WWW/IOT/IIOT</t>
+  </si>
+  <si>
+    <t>Interrobot cumminication, (voice) signal loss, multimodal communication</t>
+  </si>
+  <si>
+    <t>environment recognition, semantic functionalities,fast reaction times, GUI</t>
+  </si>
+  <si>
+    <t>N = 10</t>
   </si>
 </sst>
 </file>
@@ -587,7 +605,7 @@
   <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="18.5546875" customWidth="1"/>
+    <col min="1" max="1" width="20.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
@@ -889,15 +907,33 @@
       <c r="A13" t="s">
         <v>40</v>
       </c>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
-      <c r="J13" s="3"/>
+      <c r="B13" s="3">
+        <v>5</v>
+      </c>
+      <c r="C13" s="3">
+        <v>4</v>
+      </c>
+      <c r="D13" s="3">
+        <v>2</v>
+      </c>
+      <c r="E13" s="3">
+        <v>5</v>
+      </c>
+      <c r="F13" s="3">
+        <v>4</v>
+      </c>
+      <c r="G13" s="3">
+        <v>2</v>
+      </c>
+      <c r="H13" s="3">
+        <v>5</v>
+      </c>
+      <c r="I13" s="3">
+        <v>4</v>
+      </c>
+      <c r="J13" s="3">
+        <v>5</v>
+      </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
@@ -919,39 +955,39 @@
       </c>
       <c r="B16" s="2">
         <f>AVERAGE(B5:B14)</f>
-        <v>4.625</v>
+        <v>4.666666666666667</v>
       </c>
       <c r="C16" s="2">
         <f t="shared" ref="C16:J16" si="0">AVERAGE(C5:C14)</f>
-        <v>4.625</v>
+        <v>4.5555555555555554</v>
       </c>
       <c r="D16" s="2">
         <f t="shared" si="0"/>
-        <v>1.7142857142857142</v>
+        <v>1.75</v>
       </c>
       <c r="E16" s="2">
         <f t="shared" si="0"/>
-        <v>4.75</v>
+        <v>4.7777777777777777</v>
       </c>
       <c r="F16" s="2">
         <f t="shared" si="0"/>
-        <v>4.625</v>
+        <v>4.5555555555555554</v>
       </c>
       <c r="G16" s="2">
         <f t="shared" si="0"/>
-        <v>1.5</v>
+        <v>1.5555555555555556</v>
       </c>
       <c r="H16" s="2">
         <f t="shared" si="0"/>
-        <v>4.5</v>
+        <v>4.5555555555555554</v>
       </c>
       <c r="I16" s="2">
         <f t="shared" si="0"/>
-        <v>4.75</v>
+        <v>4.666666666666667</v>
       </c>
       <c r="J16" s="2">
         <f t="shared" si="0"/>
-        <v>4.125</v>
+        <v>4.2222222222222223</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
@@ -960,39 +996,39 @@
       </c>
       <c r="B17" s="2">
         <f>_xlfn.STDEV.S(B5:B14)</f>
-        <v>0.51754916950676566</v>
+        <v>0.5</v>
       </c>
       <c r="C17" s="2">
         <f t="shared" ref="C17:J17" si="1">_xlfn.STDEV.S(C5:C14)</f>
-        <v>0.51754916950676566</v>
+        <v>0.52704627669473059</v>
       </c>
       <c r="D17" s="2">
         <f t="shared" si="1"/>
-        <v>0.95118973121134176</v>
+        <v>0.88640526042791834</v>
       </c>
       <c r="E17" s="2">
         <f t="shared" si="1"/>
-        <v>0.46291004988627571</v>
+        <v>0.44095855184409838</v>
       </c>
       <c r="F17" s="2">
         <f t="shared" si="1"/>
-        <v>0.51754916950676566</v>
+        <v>0.52704627669473059</v>
       </c>
       <c r="G17" s="2">
         <f t="shared" si="1"/>
-        <v>0.7559289460184544</v>
+        <v>0.72648315725677881</v>
       </c>
       <c r="H17" s="2">
         <f t="shared" si="1"/>
-        <v>0.53452248382484879</v>
+        <v>0.52704627669473059</v>
       </c>
       <c r="I17" s="2">
         <f t="shared" si="1"/>
-        <v>0.46291004988627571</v>
+        <v>0.5</v>
       </c>
       <c r="J17" s="2">
         <f t="shared" si="1"/>
-        <v>1.1259916264596033</v>
+        <v>1.0929064207169994</v>
       </c>
     </row>
   </sheetData>
@@ -1006,14 +1042,14 @@
   <dimension ref="A4:D14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="46.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="40" customWidth="1"/>
+    <col min="2" max="2" width="57.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="56.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="4" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>17</v>
@@ -1127,10 +1163,25 @@
       <c r="A12" t="s">
         <v>39</v>
       </c>
+      <c r="B12" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>40</v>
+      </c>
+      <c r="B13" t="s">
+        <v>46</v>
+      </c>
+      <c r="C13" t="s">
+        <v>44</v>
+      </c>
+      <c r="D13" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
add improved yolo img, some fixes and survey eval
</commit_message>
<xml_diff>
--- a/surveyux/survey_eval.xlsx
+++ b/surveyux/survey_eval.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Githubs\IEEE-Technology-and-Society-Draft\surveyux\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66B0040B-3C9F-4803-A218-EF5876109909}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52E0AA4A-FF33-4F5E-9343-FD73A17728C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{D8488B4A-5A4F-4189-8080-6FE281BAE78B}"/>
+    <workbookView xWindow="31395" yWindow="1680" windowWidth="21600" windowHeight="11385" xr2:uid="{D8488B4A-5A4F-4189-8080-6FE281BAE78B}"/>
   </bookViews>
   <sheets>
     <sheet name="Likert Scale" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
add 2nd study, split into 2 studies, rearrange imgs and tables,
</commit_message>
<xml_diff>
--- a/surveyux/survey_eval.xlsx
+++ b/surveyux/survey_eval.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Githubs\IEEE-Technology-and-Society-Draft\surveyux\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52E0AA4A-FF33-4F5E-9343-FD73A17728C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DD16858-9C13-4893-B24F-376A4B374C01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31395" yWindow="1680" windowWidth="21600" windowHeight="11385" xr2:uid="{D8488B4A-5A4F-4189-8080-6FE281BAE78B}"/>
+    <workbookView xWindow="30660" yWindow="1830" windowWidth="21600" windowHeight="11385" activeTab="2" xr2:uid="{D8488B4A-5A4F-4189-8080-6FE281BAE78B}"/>
   </bookViews>
   <sheets>
     <sheet name="Likert Scale" sheetId="1" r:id="rId1"/>
     <sheet name="Qualitative Questions (open Qs)" sheetId="2" r:id="rId2"/>
+    <sheet name="Observer Study" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="85">
   <si>
     <t>N = 7</t>
   </si>
@@ -207,6 +208,117 @@
   </si>
   <si>
     <t>N = 10</t>
+  </si>
+  <si>
+    <t>N = 9</t>
+  </si>
+  <si>
+    <t>Only qualitative Questions</t>
+  </si>
+  <si>
+    <t>natural conversation</t>
+  </si>
+  <si>
+    <t>dynamic and safe</t>
+  </si>
+  <si>
+    <t>(retirement) home, shopping, industry</t>
+  </si>
+  <si>
+    <t>Age</t>
+  </si>
+  <si>
+    <t>Gender</t>
+  </si>
+  <si>
+    <t>m</t>
+  </si>
+  <si>
+    <t>f</t>
+  </si>
+  <si>
+    <t>accessible to people with no prior knowledge</t>
+  </si>
+  <si>
+    <t>perceived to follow without issues</t>
+  </si>
+  <si>
+    <t>home, shopping, airport, industry</t>
+  </si>
+  <si>
+    <t>conversational and able to understand</t>
+  </si>
+  <si>
+    <t>robot listens well</t>
+  </si>
+  <si>
+    <t>cleaning and transport</t>
+  </si>
+  <si>
+    <t>perceived reasonable and natural</t>
+  </si>
+  <si>
+    <t>would trust in unfimiliar surroundings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">shoppping, logistics </t>
+  </si>
+  <si>
+    <t>no: possible technical issues</t>
+  </si>
+  <si>
+    <t>transport</t>
+  </si>
+  <si>
+    <t>intuitive and natural</t>
+  </si>
+  <si>
+    <t>yes: technological progress</t>
+  </si>
+  <si>
+    <t>like a conversation with another human</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>(heavy) transport</t>
+  </si>
+  <si>
+    <t>add language options</t>
+  </si>
+  <si>
+    <t xml:space="preserve">smart navigation, but wheeled robot not suitable for every environment </t>
+  </si>
+  <si>
+    <t xml:space="preserve">stroller or transport (tools) in agriculture/gardening </t>
+  </si>
+  <si>
+    <t>safety-aware and trustworthy</t>
+  </si>
+  <si>
+    <t>Farming and last mile delivery</t>
+  </si>
+  <si>
+    <t>smoothness of the navigation</t>
+  </si>
+  <si>
+    <t>good: identification of static obstacles; questionable: dynamic obstacles?</t>
+  </si>
+  <si>
+    <t>carriying luggage</t>
+  </si>
+  <si>
+    <t>System trust</t>
+  </si>
+  <si>
+    <t>Interaction quality</t>
+  </si>
+  <si>
+    <t>Practical utility</t>
+  </si>
+  <si>
+    <t>Mean Age</t>
   </si>
 </sst>
 </file>
@@ -261,11 +373,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1039,7 +1157,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E6A12C1-567F-4693-910A-8AC58E4581FB}">
-  <dimension ref="A4:D14"/>
+  <dimension ref="A4:D13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="57.44140625" bestFit="1" customWidth="1"/>
@@ -1049,7 +1167,7 @@
   <sheetData>
     <row r="4" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>17</v>
@@ -1184,12 +1302,265 @@
         <v>45</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>41</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE6DA048-D6A6-4128-B039-7001D4F3C02C}">
+  <dimension ref="A3:G19"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="20.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="58" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="40" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="29.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="G6" s="1"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C7" s="5">
+        <v>40</v>
+      </c>
+      <c r="D7" t="s">
+        <v>50</v>
+      </c>
+      <c r="E7" t="s">
+        <v>51</v>
+      </c>
+      <c r="F7" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C8" s="5">
+        <v>38</v>
+      </c>
+      <c r="D8" t="s">
+        <v>57</v>
+      </c>
+      <c r="E8" t="s">
+        <v>58</v>
+      </c>
+      <c r="F8" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C9" s="5">
+        <v>8</v>
+      </c>
+      <c r="D9" t="s">
+        <v>60</v>
+      </c>
+      <c r="E9" t="s">
+        <v>61</v>
+      </c>
+      <c r="F9" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C10" s="5">
+        <v>39</v>
+      </c>
+      <c r="D10" t="s">
+        <v>63</v>
+      </c>
+      <c r="E10" t="s">
+        <v>64</v>
+      </c>
+      <c r="F10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C11" s="5">
+        <v>70</v>
+      </c>
+      <c r="D11" t="s">
+        <v>63</v>
+      </c>
+      <c r="E11" t="s">
+        <v>66</v>
+      </c>
+      <c r="F11" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>6</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C12" s="5">
+        <v>49</v>
+      </c>
+      <c r="D12" t="s">
+        <v>68</v>
+      </c>
+      <c r="E12" t="s">
+        <v>69</v>
+      </c>
+      <c r="F12" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>7</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C13" s="5">
+        <v>13</v>
+      </c>
+      <c r="D13" t="s">
+        <v>70</v>
+      </c>
+      <c r="E13" t="s">
+        <v>71</v>
+      </c>
+      <c r="F13" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>39</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C14" s="5">
+        <v>68</v>
+      </c>
+      <c r="D14" t="s">
+        <v>73</v>
+      </c>
+      <c r="E14" t="s">
+        <v>74</v>
+      </c>
+      <c r="F14" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>40</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C15" s="5">
+        <v>74</v>
+      </c>
+      <c r="D15" t="s">
+        <v>73</v>
+      </c>
+      <c r="E15" t="s">
+        <v>76</v>
+      </c>
+      <c r="F15" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>41</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C16" s="5">
+        <v>40</v>
+      </c>
+      <c r="D16" t="s">
+        <v>78</v>
+      </c>
+      <c r="E16" t="s">
+        <v>79</v>
+      </c>
+      <c r="F16" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="18" spans="3:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="C18" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="19" spans="3:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="C19" s="4">
+        <f>AVERAGE(C7:C16)</f>
+        <v>43.9</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>